<commit_message>
cost-cut prototype: drop N20 drivetrain, drive the 3216 kit DC motors+wheels open-loop; retune sim (0.45 m/s top, 0.10 track, 0.08 N.m torque) + BOM to ~$104
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/phase2/roybot-prototype-BOM.xlsx
+++ b/docs/phase2/roybot-prototype-BOM.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tools" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GrowBot-style first prototype (drive + chase brain + guts + portable power). Dock and cliff/bump sensors deferred to iteration 2. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have, GREY = spare. Power = 1S-&gt;TP4056-&gt;dual MT3608 (5.1V Pi / 6.0V motors). Prices are rough ballparks, not quotes.</t>
+          <t>GrowBot-style first prototype, COST-CUT: drive open-loop off the 3216 kit's own DC motors + wheels (N20s + encoders = iteration-2 upgrade). Dock + cliff/bump sensors also deferred. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have, GREY = spare. Power = 1S-&gt;TP4056-&gt;dual MT3608 (5.1V Pi / 6.0V motors). Prices are rough ballparks, not quotes.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>SUMIF(A9:A38,"Buy",H9:H38)</f>
+        <f>SUMIF(A9:A34,"Buy",H9:H34)</f>
         <v/>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="H5" s="5">
-        <f>SUMIF(A9:A38,"Have",H9:H38)+SUMIF(A9:A38,"Spare",H9:H38)</f>
+        <f>SUMIF(A9:A34,"Have",H9:H34)+SUMIF(A9:A34,"Spare",H9:H34)</f>
         <v/>
       </c>
     </row>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="H6" s="6">
-        <f>COUNTIF(A9:A38,"Print")</f>
+        <f>COUNTIF(A9:A34,"Print")</f>
         <v/>
       </c>
     </row>
@@ -642,24 +642,24 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Pololu HPCB 6V 100:1 micro metal gearmotor, EXTENDED back-shaft</t>
+          <t>TB6612FNG dual H-bridge breakout</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Verified pick (~0.75 m/s, strong torque). EXTENDED shaft is REQUIRED so the encoder mounts. Replaces the 3216's spare DC motors</t>
+          <t>Motor driver for the 3216's DC motors. VM = 6V motor rail, VCC = 3.3V, PWM &gt;=20 kHz. OPEN-LOOP (no encoders this build)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Pololu</t>
+          <t>Adafruit / Pololu</t>
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H9" s="10">
         <f>D9*G9</f>
@@ -675,12 +675,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Drivetrain</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Pololu magnetic quadrature encoder pair (micro metal gearmotor)</t>
+          <t>microSD card, 32 GB Class 10 / A1</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
@@ -688,16 +688,16 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>1200 CPR/wheel-rev at 100:1 (already x4-decoded; don't x4 again). VCC=3.3V. Closed-loop speed + odometry</t>
+          <t>NOT in your Pi kit! Raspberry Pi OS Lite 64-bit (GrowBot #2)</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Pololu</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G10" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H10" s="10">
         <f>D10*G10</f>
@@ -713,29 +713,29 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Drivetrain</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>60 mm wheel for N20 (3 mm D-shaft), rubber tire</t>
+          <t>OV5647 camera - Pi ZERO version (narrow 22-&gt;15 CSI ribbon)</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>3216 wheels don't fit the N20 shaft. Buy rubber-tired (don't print - need grip)</t>
+          <t>MUST be the Pi Zero narrow-ribbon version, NOT the standard camera ribbon (GrowBot #7)</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Pololu / Amazon</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G11" s="10" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H11" s="10">
         <f>D11*G11</f>
@@ -751,12 +751,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Drivetrain</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>TB6612FNG dual H-bridge breakout</t>
+          <t>MPU-6050 IMU (GY-521)</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
@@ -764,16 +764,16 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Motor driver. VM = 6V motor rail, VCC = 3.3V, PWM &gt;=20 kHz, encoder-static stall cutoff</t>
+          <t>Tip/stall reflexes + proprioception. I2C 0x68, 3.3V (GrowBot #6)</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Adafruit / Pololu</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" s="10">
         <f>D12*G12</f>
@@ -789,12 +789,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>microSD card, 32 GB Class 10 / A1</t>
+          <t>INMP441 I2S microphone</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>NOT in your Pi kit! Raspberry Pi OS Lite 64-bit (GrowBot #2)</t>
+          <t>Wake-word / voice in. 3.3V (GrowBot #8)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="G13" s="10" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H13" s="10">
         <f>D13*G13</f>
@@ -827,12 +827,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Sensing</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>OV5647 camera - Pi ZERO version (narrow 22-&gt;15 CSI ribbon)</t>
+          <t>MAX98357A I2S amplifier</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>MUST be the Pi Zero narrow-ribbon version, NOT the standard camera ribbon (GrowBot #7)</t>
+          <t>Speaker driver, 3.2W class-D (GrowBot #9)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H14" s="10">
         <f>D14*G14</f>
@@ -865,12 +865,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Sensing</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>MPU-6050 IMU (GY-521)</t>
+          <t>Speaker 8 ohm, 0.5-3 W (small)</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Tip/stall reflexes + proprioception. I2C 0x68, 3.3V (GrowBot #6)</t>
+          <t>Audio out (GrowBot #10)</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="G15" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H15" s="10">
         <f>D15*G15</f>
@@ -908,7 +908,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>INMP441 I2S microphone</t>
+          <t>WS2812B LED ring, 7 px, 5 V</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Wake-word / voice in. 3.3V (GrowBot #8)</t>
+          <t>Expressive 'personality' output (GrowBot #11)</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16" s="10">
         <f>D16*G16</f>
@@ -941,12 +941,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>MAX98357A I2S amplifier</t>
+          <t>18650 Li-ion cell, 2500-3500 mAh (1S)</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Speaker driver, 3.2W class-D (GrowBot #9)</t>
+          <t>Main battery. Bigger than GrowBot's 1S for N20 headroom + runtime (GrowBot #12)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="G17" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" s="10">
         <f>D17*G17</f>
@@ -979,12 +979,12 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Speaker 8 ohm, 0.5-3 W (small)</t>
+          <t>18650 battery holder</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Audio out (GrowBot #10)</t>
+          <t>Cell holder + contacts</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1017,12 +1017,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>WS2812B LED ring, 7 px, 5 V</t>
+          <t>TP4056 USB-C charge + protect module</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Expressive 'personality' output (GrowBot #11)</t>
+          <t>In-place recharging; get the PROTECTED version with OUT+/OUT- (GrowBot #13)</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G19" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H19" s="10">
         <f>D19*G19</f>
@@ -1060,15 +1060,15 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>18650 Li-ion cell, 2500-3500 mAh (1S)</t>
+          <t>MT3608 boost module (x2)</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Main battery. Bigger than GrowBot's 1S for N20 headroom + runtime (GrowBot #12)</t>
+          <t>Dual-rail: set one to ~5.1V (Pi+logic+amp+LED), one to ~6.0V (motors). Isolates Pi from motor surge; GrowBot note #5 endorses a 2nd MT3608 for motors (GrowBot #14)</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="G20" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H20" s="10">
         <f>D20*G20</f>
@@ -1098,15 +1098,15 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>18650 battery holder</t>
+          <t>Electrolytic cap 470-1000 uF, 10 V+</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Cell holder + contacts</t>
+          <t>One across each rail to cover surge dips (GrowBot #15)</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H21" s="10">
         <f>D21*G21</f>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>TP4056 USB-C charge + protect module</t>
+          <t>SPST power switch</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>In-place recharging; get the PROTECTED version with OUT+/OUT- (GrowBot #13)</t>
+          <t>Main cutoff (GrowBot #16)</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1169,20 +1169,20 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>MT3608 boost module (x2)</t>
+          <t>Hookup wire + Dupont jumpers</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Dual-rail: set one to ~5.1V (Pi+logic+amp+LED), one to ~6.0V (motors). Isolates Pi from motor surge; GrowBot note #5 endorses a 2nd MT3608 for motors (GrowBot #14)</t>
+          <t>Wire per the GrowBot diagram + the TB6612</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="G23" s="10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H23" s="10">
         <f>D23*G23</f>
@@ -1207,20 +1207,20 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Electrolytic cap 470-1000 uF, 10 V+</t>
+          <t>3M double-sided mounting squares</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>One across each rail to cover surge dips (GrowBot #15)</t>
+          <t>GrowBot's no-screw board mounting (or print mounts)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H24" s="10">
         <f>D24*G24</f>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>SPST power switch</t>
+          <t>PETG filament (known-safe), 1 spool</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Main cutoff (GrowBot #16)</t>
+          <t>For the printed parts below - skip if your printer came with filament</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="G25" s="10" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H25" s="10">
         <f>D25*G25</f>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Hookup wire + Dupont jumpers</t>
+          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
@@ -1296,16 +1296,16 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Wire per the GrowBot diagram + the TB6612</t>
+          <t>#1 cat-safety item: NO free end, over-molded. Attended play only</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>craft / Amazon</t>
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H26" s="10">
         <f>D26*G26</f>
@@ -1316,17 +1316,17 @@
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>3M double-sided mounting squares</t>
+          <t>Top cover + wheel shroud</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
@@ -1334,16 +1334,16 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>GrowBot's no-screw board mounting (or print mounts)</t>
+          <t>Cat-safety: shroud wheel gaps (&lt;4-6 mm or &gt;25 mm), cover the electronics</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G27" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H27" s="10">
         <f>D27*G27</f>
@@ -1354,17 +1354,17 @@
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>PETG filament (known-safe), 1 spool</t>
+          <t>Captive-lure boom arm</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
@@ -1372,16 +1372,16 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>For the printed parts below - skip if your printer came with filament</t>
+          <t>Rigid arm holding the lure with no free end</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H28" s="10">
         <f>D28*G28</f>
@@ -1392,17 +1392,17 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
+          <t>Battery + board mounts (optional)</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
@@ -1410,16 +1410,16 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>#1 cat-safety item: NO free end, over-molded. Attended play only</t>
+          <t>Or just use the 3M squares above</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>craft / Amazon</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H29" s="10">
         <f>D29*G29</f>
@@ -1430,30 +1430,30 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Drivetrain</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>N20 -&gt; 3216 motor-mount adapter</t>
+          <t>Raspberry Pi Zero 2 W</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>The 3216's mounts fit its DC motors, not N20s - print an adapter bracket</t>
+          <t>In your Pi kit</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>(have)</t>
         </is>
       </c>
       <c r="G30" s="10" t="n">
@@ -1468,17 +1468,17 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Top cover + wheel shroud</t>
+          <t>2x20 GPIO header</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
@@ -1486,12 +1486,12 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Cat-safety: shroud wheel gaps (&lt;4-6 mm or &gt;25 mm), cover the electronics</t>
+          <t>In your Pi kit - needs SOLDERING onto the Pi</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>(have)</t>
         </is>
       </c>
       <c r="G31" s="10" t="n">
@@ -1506,17 +1506,17 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Captive-lure boom arm</t>
+          <t>Cables incl. USB power cable</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
@@ -1524,12 +1524,12 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Rigid arm holding the lure with no free end</t>
+          <t>In your Pi kit (bench power/flashing; on-robot the Pi runs off the 5V rail)</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>(have)</t>
         </is>
       </c>
       <c r="G32" s="10" t="n">
@@ -1544,17 +1544,17 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Chassis</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Battery + board mounts (optional)</t>
+          <t>Adafruit 3216 chassis - frame + caster ball + hardware</t>
         </is>
       </c>
       <c r="D33" s="8" t="n">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Or just use the 3M squares above</t>
+          <t>Your base kit = the robot body</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>(have)</t>
         </is>
       </c>
       <c r="G33" s="10" t="n">
@@ -1587,12 +1587,12 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Raspberry Pi Zero 2 W</t>
+          <t>3216 DC motors + 2 wheels (USED this build)</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>In your Pi kit</t>
+          <t>Drive open-loop off these instead of buying N20s. No encoders -&gt; no odometry/closed-loop speed (fine for an attended prototype). N20 + encoder = iteration-2 upgrade</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -1617,165 +1617,13 @@
       </c>
       <c r="I34" s="8" t="inlineStr"/>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>Have</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>2x20 GPIO header</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>In your Pi kit - needs SOLDERING onto the Pi</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>(have)</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="10">
-        <f>D35*G35</f>
-        <v/>
-      </c>
-      <c r="I35" s="8" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Have</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Cables incl. USB power cable</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>In your Pi kit (bench power/flashing; on-robot the Pi runs off the 5V rail)</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>(have)</t>
-        </is>
-      </c>
-      <c r="G36" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="10">
-        <f>D36*G36</f>
-        <v/>
-      </c>
-      <c r="I36" s="8" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Have</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>Chassis</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Adafruit 3216 chassis - frame + caster ball + hardware</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>Your base kit = the robot body</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>(have)</t>
-        </is>
-      </c>
-      <c r="G37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="10">
-        <f>D37*G37</f>
-        <v/>
-      </c>
-      <c r="I37" s="8" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>Spare</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Chassis</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>3216 bundled DC motors + 2 wheels</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>Superseded by the N20 drivetrain - keep as spares</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>(have)</t>
-        </is>
-      </c>
-      <c r="G38" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="10">
-        <f>D38*G38</f>
-        <v/>
-      </c>
-      <c r="I38" s="8" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A8:I38"/>
+  <autoFilter ref="A8:I34"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A9:A38">
+  <conditionalFormatting sqref="A9:A34">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Buy"</formula>
     </cfRule>
@@ -1790,7 +1638,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A9:A38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A9:A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Buy,Print,Have,Spare"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
power: single 5V rail (drop the 6V N20 leftover) - one MT3608 boost feeds Pi + 3216 DC motors at 5V; BOM ~$101
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/phase2/roybot-prototype-BOM.xlsx
+++ b/docs/phase2/roybot-prototype-BOM.xlsx
@@ -545,7 +545,7 @@
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GrowBot-style first prototype, COST-CUT: drive open-loop off the 3216 kit's own DC motors + wheels (N20s + encoders = iteration-2 upgrade). Dock + cliff/bump sensors also deferred. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have, GREY = spare. Power = 1S-&gt;TP4056-&gt;dual MT3608 (5.1V Pi / 6.0V motors). Prices are rough ballparks, not quotes.</t>
+          <t>GrowBot-style first prototype, COST-CUT: drive open-loop off the 3216 kit's own DC motors + wheels (N20s + encoders = iteration-2 upgrade). Dock + cliff/bump sensors also deferred. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have. Power = 1S 18650 -&gt; TP4056 -&gt; single MT3608 (one ~5.1V rail for everything; 3216 motors are 3-6V). Prices are rough ballparks, not quotes.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Motor driver for the 3216's DC motors. VM = 6V motor rail, VCC = 3.3V, PWM &gt;=20 kHz. OPEN-LOOP (no encoders this build)</t>
+          <t>Motor driver for the 3216's DC motors. VM = the shared 5V rail, VCC = 3.3V, PWM &gt;=20 kHz. OPEN-LOOP (no encoders this build)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Main battery. Bigger than GrowBot's 1S for N20 headroom + runtime (GrowBot #12)</t>
+          <t>Main battery (you don't have one). GrowBot uses 800-1200 mAh; a 2500-3500 mAh 18650 gives more runtime (GrowBot #12)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1060,15 +1060,15 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>MT3608 boost module (x2)</t>
+          <t>MT3608 boost module</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Dual-rail: set one to ~5.1V (Pi+logic+amp+LED), one to ~6.0V (motors). Isolates Pi from motor surge; GrowBot note #5 endorses a 2nd MT3608 for motors (GrowBot #14)</t>
+          <t>Boosts the 1S cell (3.7V) UP to ~5.1V = the single shared 5V rail (Pi + motors + amp + LED), GrowBot V0 style. 3216 motors are 3-6V so 5V is fine (dial to 6V for max speed if ever wanted). Add a 2nd MT3608 for a separate motor rail ONLY if a double-stall reboots the Pi (GrowBot #14)</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1102,11 +1102,11 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>One across each rail to cover surge dips (GrowBot #15)</t>
+          <t>Across the 5V rail to cover motor surge dips (GrowBot #15)</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">

</xml_diff>

<commit_message>
restore N20+encoder drivetrain: closed-loop fixes open-loop sim2real risk + enables stall cutoff/odometry; dual 5.1V/6V rail; sim back to N20 envelope (final_policy matches, no retrain); +WS2812 resistor; BOM ~$158
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/phase2/roybot-prototype-BOM.xlsx
+++ b/docs/phase2/roybot-prototype-BOM.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tools" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$8:$I$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GrowBot-style first prototype, COST-CUT: drive open-loop off the 3216 kit's own DC motors + wheels (N20s + encoders = iteration-2 upgrade). Dock + cliff/bump sensors also deferred. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have. Power = 1S 18650 -&gt; TP4056 -&gt; single MT3608 (one ~5.1V rail for everything; 3216 motors are 3-6V). Prices are rough ballparks, not quotes.</t>
+          <t>GrowBot-style first prototype: N20 + encoder closed-loop drivetrain (enables stall cutoff + odometry) + full GrowBot senses (camera + mic + speaker + IMU + LED). Dock + cliff/bump sensors deferred to iteration 2. RED = buy (your shopping list), BLUE = 3D-print, GREEN = already have, GREY = spare. Power = 1S 18650 -&gt; TP4056 -&gt; dual MT3608 (~5.1V Pi rail + ~6.0V motor rail). Tools assumed on hand. Prices are rough ballparks, not quotes.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>SUMIF(A9:A34,"Buy",H9:H34)</f>
+        <f>SUMIF(A9:A39,"Buy",H9:H39)</f>
         <v/>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="H5" s="5">
-        <f>SUMIF(A9:A34,"Have",H9:H34)+SUMIF(A9:A34,"Spare",H9:H34)</f>
+        <f>SUMIF(A9:A39,"Have",H9:H39)+SUMIF(A9:A39,"Spare",H9:H39)</f>
         <v/>
       </c>
     </row>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="H6" s="6">
-        <f>COUNTIF(A9:A34,"Print")</f>
+        <f>COUNTIF(A9:A39,"Print")</f>
         <v/>
       </c>
     </row>
@@ -642,24 +642,24 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>TB6612FNG dual H-bridge breakout</t>
+          <t>Pololu HPCB 6V 100:1 micro metal gearmotor, EXTENDED back-shaft</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Motor driver for the 3216's DC motors. VM = the shared 5V rail, VCC = 3.3V, PWM &gt;=20 kHz. OPEN-LOOP (no encoders this build)</t>
+          <t>Verified pick (~0.75 m/s, strong torque). EXTENDED shaft is REQUIRED so the encoder mounts. Replaces the 3216's DC motors (now spares)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Adafruit / Pololu</t>
+          <t>Pololu</t>
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H9" s="10">
         <f>D9*G9</f>
@@ -675,12 +675,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>microSD card, 32 GB Class 10 / A1</t>
+          <t>Pololu magnetic quadrature encoder pair (micro metal gearmotor)</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
@@ -688,16 +688,16 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>NOT in your Pi kit! Raspberry Pi OS Lite 64-bit (GrowBot #2)</t>
+          <t>1200 CPR/wheel-rev at 100:1 (already x4-decoded). VCC=3.3V. Gives closed-loop wheel speed (matches the sim's velocity model), encoder-vs-command STALL CUTOFF, and odometry for docking</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Pololu</t>
         </is>
       </c>
       <c r="G10" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H10" s="10">
         <f>D10*G10</f>
@@ -713,29 +713,29 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Sensing</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>OV5647 camera - Pi ZERO version (narrow 22-&gt;15 CSI ribbon)</t>
+          <t>60 mm wheel for N20 (3 mm D-shaft), rubber tire</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>MUST be the Pi Zero narrow-ribbon version, NOT the standard camera ribbon (GrowBot #7)</t>
+          <t>3216 wheels don't fit the N20 shaft. Rubber tire for grip</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Pololu / Amazon</t>
         </is>
       </c>
       <c r="G11" s="10" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H11" s="10">
         <f>D11*G11</f>
@@ -751,12 +751,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Sensing</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>MPU-6050 IMU (GY-521)</t>
+          <t>TB6612FNG dual H-bridge breakout</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
@@ -764,16 +764,16 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Tip/stall reflexes + proprioception. I2C 0x68, 3.3V (GrowBot #6)</t>
+          <t>Motor driver. VM = the 6V motor rail, VCC = 3.3V, PWM &gt;=20 kHz. Closed-loop via the encoders + firmware stall cutoff</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Adafruit / Pololu</t>
         </is>
       </c>
       <c r="G12" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" s="10">
         <f>D12*G12</f>
@@ -789,12 +789,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>INMP441 I2S microphone</t>
+          <t>microSD card, 32 GB Class 10 / A1</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
@@ -802,7 +802,7 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Wake-word / voice in. 3.3V (GrowBot #8)</t>
+          <t>NOT in your Pi kit! Raspberry Pi OS Lite 64-bit (GrowBot #2)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="G13" s="10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H13" s="10">
         <f>D13*G13</f>
@@ -827,12 +827,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>MAX98357A I2S amplifier</t>
+          <t>OV5647 camera - Pi ZERO version (narrow 22-&gt;15 CSI ribbon)</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
@@ -840,7 +840,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Speaker driver, 3.2W class-D (GrowBot #9)</t>
+          <t>MUST be the Pi Zero narrow-ribbon version, NOT the standard camera ribbon (GrowBot #7)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H14" s="10">
         <f>D14*G14</f>
@@ -865,12 +865,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Voice/Lights</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Speaker 8 ohm, 0.5-3 W (small)</t>
+          <t>MPU-6050 IMU (GY-521)</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Audio out (GrowBot #10)</t>
+          <t>Tip/stall reflexes + proprioception. I2C 0x68, 3.3V (GrowBot #6)</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="G15" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H15" s="10">
         <f>D15*G15</f>
@@ -908,7 +908,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>WS2812B LED ring, 7 px, 5 V</t>
+          <t>INMP441 I2S microphone</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Expressive 'personality' output (GrowBot #11)</t>
+          <t>Wake-word / voice in. 3.3V (GrowBot #8)</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16" s="10">
         <f>D16*G16</f>
@@ -941,12 +941,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>18650 Li-ion cell, 2500-3500 mAh (1S)</t>
+          <t>MAX98357A I2S amplifier</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
@@ -954,7 +954,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Main battery (you don't have one). GrowBot uses 800-1200 mAh; a 2500-3500 mAh 18650 gives more runtime (GrowBot #12)</t>
+          <t>Speaker driver, 3.2W class-D (GrowBot #9)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="G17" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H17" s="10">
         <f>D17*G17</f>
@@ -979,12 +979,12 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>18650 battery holder</t>
+          <t>Speaker 8 ohm, 0.5-3 W (small)</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Cell holder + contacts</t>
+          <t>Audio out (GrowBot #10)</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1017,12 +1017,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Voice/Lights</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>TP4056 USB-C charge + protect module</t>
+          <t>WS2812B LED ring, 7 px, 5 V</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>In-place recharging; get the PROTECTED version with OUT+/OUT- (GrowBot #13)</t>
+          <t>Expressive 'personality' output (GrowBot #11)</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G19" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H19" s="10">
         <f>D19*G19</f>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>MT3608 boost module</t>
+          <t>18650 Li-ion cell, 2500-3500 mAh (1S)</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Boosts the 1S cell (3.7V) UP to ~5.1V = the single shared 5V rail (Pi + motors + amp + LED), GrowBot V0 style. 3216 motors are 3-6V so 5V is fine (dial to 6V for max speed if ever wanted). Add a 2nd MT3608 for a separate motor rail ONLY if a double-stall reboots the Pi (GrowBot #14)</t>
+          <t>Main battery (you don't have one). GrowBot uses 800-1200 mAh; a 2500-3500 mAh 18650 gives more runtime (GrowBot #12)</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="G20" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H20" s="10">
         <f>D20*G20</f>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Electrolytic cap 470-1000 uF, 10 V+</t>
+          <t>18650 battery holder</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Across the 5V rail to cover motor surge dips (GrowBot #15)</t>
+          <t>Cell holder + contacts</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="10">
         <f>D21*G21</f>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>SPST power switch</t>
+          <t>TP4056 USB-C charge + protect module</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Main cutoff (GrowBot #16)</t>
+          <t>In-place recharging; get the PROTECTED version with OUT+/OUT- (GrowBot #13)</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1169,20 +1169,20 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Hookup wire + Dupont jumpers</t>
+          <t>MT3608 boost module (x2)</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Wire per the GrowBot diagram + the TB6612</t>
+          <t>Dual-rail off the 1S cell: one set to ~5.1V (Pi + amp + LED), one to ~6.0V (the N20 motor rail = TB6612 VM). A separate motor rail isolates the Pi from motor surge/stall brownout - needed given the N20s' 1.5A stall (GrowBot note #5 endorses a 2nd MT3608 for motors)</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="G23" s="10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H23" s="10">
         <f>D23*G23</f>
@@ -1207,20 +1207,20 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>3M double-sided mounting squares</t>
+          <t>Electrolytic cap 470-1000 uF, 10 V+</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>GrowBot's no-screw board mounting (or print mounts)</t>
+          <t>One across each rail for surge dips; pair with firmware PWM soft-start + a drive watchdog (GrowBot #15)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H24" s="10">
         <f>D24*G24</f>
@@ -1245,12 +1245,12 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>PETG filament (known-safe), 1 spool</t>
+          <t>SPST power switch</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>For the printed parts below - skip if your printer came with filament</t>
+          <t>Main cutoff (GrowBot #16)</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="G25" s="10" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H25" s="10">
         <f>D25*G25</f>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
+          <t>Hookup wire + Dupont jumpers</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
@@ -1296,16 +1296,16 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>#1 cat-safety item: NO free end, over-molded. Attended play only</t>
+          <t>Wire per the GrowBot diagram + the TB6612</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>craft / Amazon</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H26" s="10">
         <f>D26*G26</f>
@@ -1316,17 +1316,17 @@
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Top cover + wheel shroud</t>
+          <t>330-470 ohm resistor (WS2812 data line)</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
@@ -1334,16 +1334,16 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Cat-safety: shroud wheel gaps (&lt;4-6 mm or &gt;25 mm), cover the electronics</t>
+          <t>Series resistor on the LED-ring data line (3.3V GPIO -&gt; 5V ring); reality-check fix</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G27" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" s="10">
         <f>D27*G27</f>
@@ -1354,17 +1354,17 @@
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Captive-lure boom arm</t>
+          <t>3M double-sided mounting squares</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
@@ -1372,16 +1372,16 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Rigid arm holding the lure with no free end</t>
+          <t>GrowBot's no-screw board mounting (or print mounts)</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H28" s="10">
         <f>D28*G28</f>
@@ -1392,17 +1392,17 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Battery + board mounts (optional)</t>
+          <t>PETG filament (known-safe), 1 spool</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
@@ -1410,16 +1410,16 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Or just use the 3M squares above</t>
+          <t>For the printed parts below - skip if your printer came with filament</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H29" s="10">
         <f>D29*G29</f>
@@ -1430,17 +1430,17 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Have</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Raspberry Pi Zero 2 W</t>
+          <t>Captive lure (feather/pom on short rigid/braided arm)</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
@@ -1448,16 +1448,16 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>In your Pi kit</t>
+          <t>#1 cat-safety item: NO free end, over-molded. Attended play only</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>(have)</t>
+          <t>craft / Amazon</t>
         </is>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H30" s="10">
         <f>D30*G30</f>
@@ -1468,30 +1468,30 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Have</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Drivetrain</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>2x20 GPIO header</t>
+          <t>N20 -&gt; 3216 motor-mount adapter</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>In your Pi kit - needs SOLDERING onto the Pi</t>
+          <t>The 3216's mounts fit its DC motors, not N20s - print an adapter bracket</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>(have)</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G31" s="10" t="n">
@@ -1506,17 +1506,17 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Have</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Cables incl. USB power cable</t>
+          <t>Top cover + wheel shroud</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
@@ -1524,12 +1524,12 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>In your Pi kit (bench power/flashing; on-robot the Pi runs off the 5V rail)</t>
+          <t>Cat-safety: shroud wheel gaps (&lt;4-6 mm or &gt;25 mm), cover the electronics</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>(have)</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G32" s="10" t="n">
@@ -1544,17 +1544,17 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Have</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Chassis</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Adafruit 3216 chassis - frame + caster ball + hardware</t>
+          <t>Captive-lure boom arm</t>
         </is>
       </c>
       <c r="D33" s="8" t="n">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Your base kit = the robot body</t>
+          <t>Rigid arm holding the lure with no free end</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>(have)</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G33" s="10" t="n">
@@ -1582,17 +1582,17 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Have</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Drivetrain</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>3216 DC motors + 2 wheels (USED this build)</t>
+          <t>Battery + board mounts (optional)</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Drive open-loop off these instead of buying N20s. No encoders -&gt; no odometry/closed-loop speed (fine for an attended prototype). N20 + encoder = iteration-2 upgrade</t>
+          <t>Or just use the 3M squares above</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>(have)</t>
+          <t>3D print</t>
         </is>
       </c>
       <c r="G34" s="10" t="n">
@@ -1617,13 +1617,203 @@
       </c>
       <c r="I34" s="8" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Raspberry Pi Zero 2 W</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>In your Pi kit</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>(have)</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10">
+        <f>D35*G35</f>
+        <v/>
+      </c>
+      <c r="I35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>2x20 GPIO header</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>In your Pi kit - needs SOLDERING onto the Pi</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>(have)</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="10">
+        <f>D36*G36</f>
+        <v/>
+      </c>
+      <c r="I36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Cables incl. USB power cable</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>In your Pi kit (bench power/flashing; on-robot the Pi runs off the 5V rail)</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>(have)</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="10">
+        <f>D37*G37</f>
+        <v/>
+      </c>
+      <c r="I37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Have</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Chassis</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit 3216 chassis - frame + caster ball + hardware</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Your base kit = the robot body</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>(have)</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="10">
+        <f>D38*G38</f>
+        <v/>
+      </c>
+      <c r="I38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Spare</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Drivetrain</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>3216 DC motors + 2 wheels</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Superseded by the N20 + encoder drivetrain - keep as spares / backup</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>(have)</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="10">
+        <f>D39*G39</f>
+        <v/>
+      </c>
+      <c r="I39" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I34"/>
+  <autoFilter ref="A8:I39"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A9:A34">
+  <conditionalFormatting sqref="A9:A39">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Buy"</formula>
     </cfRule>
@@ -1638,7 +1828,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A9:A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A9:A39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Buy,Print,Have,Spare"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>